<commit_message>
Update model and results files with new training and validation data
- Updated the FaultSeg3D_BEST.pth model file with improved weights.
- Revised training results in train_result.xlsx and val_result.xlsx to reflect the latest training metrics.
- Modified valid_final_result.txt to include updated validation metrics:
  - New valid loss: 0.6353
  - New valid IoU: 0.7949
  - New valid Dice: 0.8758
</commit_message>
<xml_diff>
--- a/EXP/1300_50_FFCUnet/results/train/train_result.xlsx
+++ b/EXP/1300_50_FFCUnet/results/train/train_result.xlsx
@@ -450,13 +450,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1.40966</v>
+        <v>1.41063</v>
       </c>
       <c r="C2" t="n">
-        <v>0.27481</v>
+        <v>0.34811</v>
       </c>
       <c r="D2" t="n">
-        <v>0.40769</v>
+        <v>0.47858</v>
       </c>
     </row>
     <row r="3">
@@ -464,13 +464,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.2998</v>
+        <v>1.29198</v>
       </c>
       <c r="C3" t="n">
-        <v>0.36496</v>
+        <v>0.46931</v>
       </c>
       <c r="D3" t="n">
-        <v>0.50749</v>
+        <v>0.60058</v>
       </c>
     </row>
     <row r="4">
@@ -478,13 +478,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.23903</v>
+        <v>1.22891</v>
       </c>
       <c r="C4" t="n">
-        <v>0.40713</v>
+        <v>0.51203</v>
       </c>
       <c r="D4" t="n">
-        <v>0.54872</v>
+        <v>0.64095</v>
       </c>
     </row>
     <row r="5">
@@ -492,13 +492,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.18789</v>
+        <v>1.1769</v>
       </c>
       <c r="C5" t="n">
-        <v>0.44888</v>
+        <v>0.54611</v>
       </c>
       <c r="D5" t="n">
-        <v>0.58793</v>
+        <v>0.67235</v>
       </c>
     </row>
     <row r="6">
@@ -506,13 +506,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.1428</v>
+        <v>1.12759</v>
       </c>
       <c r="C6" t="n">
-        <v>0.49517</v>
+        <v>0.5736</v>
       </c>
       <c r="D6" t="n">
-        <v>0.63004</v>
+        <v>0.69735</v>
       </c>
     </row>
     <row r="7">
@@ -520,13 +520,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.09709</v>
+        <v>1.08107</v>
       </c>
       <c r="C7" t="n">
-        <v>0.53404</v>
+        <v>0.59712</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6649</v>
+        <v>0.71853</v>
       </c>
     </row>
     <row r="8">
@@ -534,13 +534,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.05589</v>
+        <v>1.0398</v>
       </c>
       <c r="C8" t="n">
-        <v>0.56604</v>
+        <v>0.61564</v>
       </c>
       <c r="D8" t="n">
-        <v>0.69311</v>
+        <v>0.73476</v>
       </c>
     </row>
     <row r="9">
@@ -548,13 +548,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.01631</v>
+        <v>1.00327</v>
       </c>
       <c r="C9" t="n">
-        <v>0.59426</v>
+        <v>0.63125</v>
       </c>
       <c r="D9" t="n">
-        <v>0.71771</v>
+        <v>0.74826</v>
       </c>
     </row>
     <row r="10">
@@ -562,13 +562,13 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>0.97663</v>
+        <v>0.96529</v>
       </c>
       <c r="C10" t="n">
-        <v>0.6408199999999999</v>
+        <v>0.64724</v>
       </c>
       <c r="D10" t="n">
-        <v>0.75715</v>
+        <v>0.762</v>
       </c>
     </row>
     <row r="11">
@@ -576,13 +576,13 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>0.94324</v>
+        <v>0.93352</v>
       </c>
       <c r="C11" t="n">
-        <v>0.66083</v>
+        <v>0.65906</v>
       </c>
       <c r="D11" t="n">
-        <v>0.77382</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="12">
@@ -590,13 +590,13 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>0.91356</v>
+        <v>0.90513</v>
       </c>
       <c r="C12" t="n">
-        <v>0.67216</v>
+        <v>0.67013</v>
       </c>
       <c r="D12" t="n">
-        <v>0.7832</v>
+        <v>0.78122</v>
       </c>
     </row>
     <row r="13">
@@ -604,13 +604,13 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>0.88715</v>
+        <v>0.88305</v>
       </c>
       <c r="C13" t="n">
-        <v>0.68213</v>
+        <v>0.67764</v>
       </c>
       <c r="D13" t="n">
-        <v>0.79133</v>
+        <v>0.78733</v>
       </c>
     </row>
     <row r="14">
@@ -618,13 +618,13 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>0.85902</v>
+        <v>0.85567</v>
       </c>
       <c r="C14" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.68808</v>
       </c>
       <c r="D14" t="n">
-        <v>0.80021</v>
+        <v>0.79598</v>
       </c>
     </row>
     <row r="15">
@@ -632,13 +632,13 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>0.83777</v>
+        <v>0.83757</v>
       </c>
       <c r="C15" t="n">
-        <v>0.69998</v>
+        <v>0.6946600000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8058</v>
+        <v>0.80131</v>
       </c>
     </row>
     <row r="16">
@@ -646,13 +646,13 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>0.81545</v>
+        <v>0.8173899999999999</v>
       </c>
       <c r="C16" t="n">
-        <v>0.70801</v>
+        <v>0.70259</v>
       </c>
       <c r="D16" t="n">
-        <v>0.81221</v>
+        <v>0.80771</v>
       </c>
     </row>
     <row r="17">
@@ -660,13 +660,13 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>0.8048999999999999</v>
+        <v>0.80228</v>
       </c>
       <c r="C17" t="n">
-        <v>0.71131</v>
+        <v>0.70825</v>
       </c>
       <c r="D17" t="n">
-        <v>0.81475</v>
+        <v>0.81221</v>
       </c>
     </row>
     <row r="18">
@@ -674,13 +674,13 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>0.78684</v>
+        <v>0.78623</v>
       </c>
       <c r="C18" t="n">
-        <v>0.7176900000000001</v>
+        <v>0.71468</v>
       </c>
       <c r="D18" t="n">
-        <v>0.8198</v>
+        <v>0.81736</v>
       </c>
     </row>
     <row r="19">
@@ -688,13 +688,13 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>0.77332</v>
+        <v>0.7723</v>
       </c>
       <c r="C19" t="n">
-        <v>0.72263</v>
+        <v>0.72016</v>
       </c>
       <c r="D19" t="n">
-        <v>0.8237</v>
+        <v>0.8217</v>
       </c>
     </row>
     <row r="20">
@@ -702,13 +702,13 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>0.76411</v>
+        <v>0.76616</v>
       </c>
       <c r="C20" t="n">
-        <v>0.72556</v>
+        <v>0.72216</v>
       </c>
       <c r="D20" t="n">
-        <v>0.82596</v>
+        <v>0.8232</v>
       </c>
     </row>
     <row r="21">
@@ -716,13 +716,13 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>0.74901</v>
+        <v>0.7583800000000001</v>
       </c>
       <c r="C21" t="n">
-        <v>0.73163</v>
+        <v>0.72487</v>
       </c>
       <c r="D21" t="n">
-        <v>0.83072</v>
+        <v>0.82534</v>
       </c>
     </row>
     <row r="22">
@@ -730,13 +730,13 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>0.73932</v>
+        <v>0.74799</v>
       </c>
       <c r="C22" t="n">
-        <v>0.73552</v>
+        <v>0.72949</v>
       </c>
       <c r="D22" t="n">
-        <v>0.83371</v>
+        <v>0.8289299999999999</v>
       </c>
     </row>
     <row r="23">
@@ -744,13 +744,13 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>0.73243</v>
+        <v>0.73794</v>
       </c>
       <c r="C23" t="n">
-        <v>0.73825</v>
+        <v>0.73362</v>
       </c>
       <c r="D23" t="n">
-        <v>0.83579</v>
+        <v>0.83217</v>
       </c>
     </row>
     <row r="24">
@@ -758,13 +758,13 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>0.72336</v>
+        <v>0.7307</v>
       </c>
       <c r="C24" t="n">
-        <v>0.74153</v>
+        <v>0.73672</v>
       </c>
       <c r="D24" t="n">
-        <v>0.83834</v>
+        <v>0.8345399999999999</v>
       </c>
     </row>
     <row r="25">
@@ -772,13 +772,13 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>0.72117</v>
+        <v>0.7248</v>
       </c>
       <c r="C25" t="n">
-        <v>0.74208</v>
+        <v>0.7391</v>
       </c>
       <c r="D25" t="n">
-        <v>0.83873</v>
+        <v>0.8364</v>
       </c>
     </row>
     <row r="26">
@@ -786,13 +786,13 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>0.7135899999999999</v>
+        <v>0.72066</v>
       </c>
       <c r="C26" t="n">
-        <v>0.7454499999999999</v>
+        <v>0.74091</v>
       </c>
       <c r="D26" t="n">
-        <v>0.84127</v>
+        <v>0.83774</v>
       </c>
     </row>
     <row r="27">
@@ -800,13 +800,13 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>0.70788</v>
+        <v>0.71217</v>
       </c>
       <c r="C27" t="n">
-        <v>0.74776</v>
+        <v>0.74473</v>
       </c>
       <c r="D27" t="n">
-        <v>0.84305</v>
+        <v>0.84071</v>
       </c>
     </row>
     <row r="28">
@@ -814,13 +814,13 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>0.70386</v>
+        <v>0.70901</v>
       </c>
       <c r="C28" t="n">
-        <v>0.74925</v>
+        <v>0.74587</v>
       </c>
       <c r="D28" t="n">
-        <v>0.84414</v>
+        <v>0.84156</v>
       </c>
     </row>
     <row r="29">
@@ -828,13 +828,13 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>0.70289</v>
+        <v>0.70169</v>
       </c>
       <c r="C29" t="n">
-        <v>0.74965</v>
+        <v>0.74922</v>
       </c>
       <c r="D29" t="n">
-        <v>0.84444</v>
+        <v>0.84412</v>
       </c>
     </row>
     <row r="30">
@@ -842,13 +842,13 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>0.69435</v>
+        <v>0.70103</v>
       </c>
       <c r="C30" t="n">
-        <v>0.7535500000000001</v>
+        <v>0.74973</v>
       </c>
       <c r="D30" t="n">
-        <v>0.8474</v>
+        <v>0.84448</v>
       </c>
     </row>
     <row r="31">
@@ -856,13 +856,13 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>0.68948</v>
+        <v>0.69408</v>
       </c>
       <c r="C31" t="n">
-        <v>0.7555500000000001</v>
+        <v>0.7528899999999999</v>
       </c>
       <c r="D31" t="n">
-        <v>0.8489100000000001</v>
+        <v>0.84688</v>
       </c>
     </row>
     <row r="32">
@@ -870,13 +870,13 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>0.68645</v>
+        <v>0.6897</v>
       </c>
       <c r="C32" t="n">
-        <v>0.7569</v>
+        <v>0.75519</v>
       </c>
       <c r="D32" t="n">
-        <v>0.84992</v>
+        <v>0.84861</v>
       </c>
     </row>
     <row r="33">
@@ -884,13 +884,13 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>0.68662</v>
+        <v>0.68982</v>
       </c>
       <c r="C33" t="n">
-        <v>0.75664</v>
+        <v>0.75467</v>
       </c>
       <c r="D33" t="n">
-        <v>0.8496899999999999</v>
+        <v>0.84822</v>
       </c>
     </row>
     <row r="34">
@@ -898,13 +898,13 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>0.68118</v>
+        <v>0.6839</v>
       </c>
       <c r="C34" t="n">
-        <v>0.75932</v>
+        <v>0.75773</v>
       </c>
       <c r="D34" t="n">
-        <v>0.85173</v>
+        <v>0.85051</v>
       </c>
     </row>
     <row r="35">
@@ -912,13 +912,13 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>0.6752</v>
+        <v>0.68435</v>
       </c>
       <c r="C35" t="n">
-        <v>0.76208</v>
+        <v>0.75751</v>
       </c>
       <c r="D35" t="n">
-        <v>0.8538</v>
+        <v>0.85032</v>
       </c>
     </row>
     <row r="36">
@@ -926,13 +926,13 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>0.6738</v>
+        <v>0.67991</v>
       </c>
       <c r="C36" t="n">
-        <v>0.76276</v>
+        <v>0.75968</v>
       </c>
       <c r="D36" t="n">
-        <v>0.85432</v>
+        <v>0.8519600000000001</v>
       </c>
     </row>
     <row r="37">
@@ -940,13 +940,13 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>0.67015</v>
+        <v>0.67523</v>
       </c>
       <c r="C37" t="n">
-        <v>0.76466</v>
+        <v>0.76201</v>
       </c>
       <c r="D37" t="n">
-        <v>0.8557</v>
+        <v>0.8536899999999999</v>
       </c>
     </row>
     <row r="38">
@@ -954,13 +954,13 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>0.66687</v>
+        <v>0.6732900000000001</v>
       </c>
       <c r="C38" t="n">
-        <v>0.7662600000000001</v>
+        <v>0.7630400000000001</v>
       </c>
       <c r="D38" t="n">
-        <v>0.85688</v>
+        <v>0.85446</v>
       </c>
     </row>
     <row r="39">
@@ -968,13 +968,13 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>0.66477</v>
+        <v>0.66723</v>
       </c>
       <c r="C39" t="n">
-        <v>0.76702</v>
+        <v>0.766</v>
       </c>
       <c r="D39" t="n">
-        <v>0.85745</v>
+        <v>0.85667</v>
       </c>
     </row>
     <row r="40">
@@ -982,13 +982,13 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>0.6626</v>
+        <v>0.66679</v>
       </c>
       <c r="C40" t="n">
-        <v>0.76841</v>
+        <v>0.76631</v>
       </c>
       <c r="D40" t="n">
-        <v>0.85847</v>
+        <v>0.85689</v>
       </c>
     </row>
     <row r="41">
@@ -996,13 +996,13 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>0.66306</v>
+        <v>0.66735</v>
       </c>
       <c r="C41" t="n">
-        <v>0.76811</v>
+        <v>0.76586</v>
       </c>
       <c r="D41" t="n">
-        <v>0.85824</v>
+        <v>0.85655</v>
       </c>
     </row>
     <row r="42">
@@ -1010,13 +1010,13 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>0.65573</v>
+        <v>0.66378</v>
       </c>
       <c r="C42" t="n">
-        <v>0.7718699999999999</v>
+        <v>0.76783</v>
       </c>
       <c r="D42" t="n">
-        <v>0.8610100000000001</v>
+        <v>0.8580100000000001</v>
       </c>
     </row>
     <row r="43">
@@ -1024,13 +1024,13 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>0.65713</v>
+        <v>0.65816</v>
       </c>
       <c r="C43" t="n">
-        <v>0.77088</v>
+        <v>0.77062</v>
       </c>
       <c r="D43" t="n">
-        <v>0.86027</v>
+        <v>0.86007</v>
       </c>
     </row>
     <row r="44">
@@ -1038,13 +1038,13 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>0.6562</v>
+        <v>0.65574</v>
       </c>
       <c r="C44" t="n">
-        <v>0.7711</v>
+        <v>0.77173</v>
       </c>
       <c r="D44" t="n">
-        <v>0.86044</v>
+        <v>0.86091</v>
       </c>
     </row>
     <row r="45">
@@ -1052,13 +1052,13 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>0.64895</v>
+        <v>0.65363</v>
       </c>
       <c r="C45" t="n">
-        <v>0.7752</v>
+        <v>0.77322</v>
       </c>
       <c r="D45" t="n">
-        <v>0.8634500000000001</v>
+        <v>0.86197</v>
       </c>
     </row>
     <row r="46">
@@ -1066,13 +1066,13 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>0.65133</v>
+        <v>0.65246</v>
       </c>
       <c r="C46" t="n">
-        <v>0.77437</v>
+        <v>0.77351</v>
       </c>
       <c r="D46" t="n">
-        <v>0.86281</v>
+        <v>0.86219</v>
       </c>
     </row>
     <row r="47">
@@ -1080,13 +1080,13 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>0.6503100000000001</v>
+        <v>0.64979</v>
       </c>
       <c r="C47" t="n">
-        <v>0.77452</v>
+        <v>0.77497</v>
       </c>
       <c r="D47" t="n">
-        <v>0.86293</v>
+        <v>0.86324</v>
       </c>
     </row>
     <row r="48">
@@ -1094,13 +1094,13 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>0.6444299999999999</v>
+        <v>0.64701</v>
       </c>
       <c r="C48" t="n">
-        <v>0.7776</v>
+        <v>0.77658</v>
       </c>
       <c r="D48" t="n">
-        <v>0.8652</v>
+        <v>0.86443</v>
       </c>
     </row>
     <row r="49">
@@ -1108,13 +1108,13 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>0.64489</v>
+        <v>0.64781</v>
       </c>
       <c r="C49" t="n">
-        <v>0.77744</v>
+        <v>0.77615</v>
       </c>
       <c r="D49" t="n">
-        <v>0.86507</v>
+        <v>0.86411</v>
       </c>
     </row>
     <row r="50">
@@ -1122,13 +1122,13 @@
         <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>0.64229</v>
+        <v>0.64495</v>
       </c>
       <c r="C50" t="n">
-        <v>0.77882</v>
+        <v>0.77747</v>
       </c>
       <c r="D50" t="n">
-        <v>0.8660600000000001</v>
+        <v>0.86507</v>
       </c>
     </row>
     <row r="51">
@@ -1136,13 +1136,13 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>0.64122</v>
+        <v>0.64051</v>
       </c>
       <c r="C51" t="n">
-        <v>0.77943</v>
+        <v>0.78001</v>
       </c>
       <c r="D51" t="n">
-        <v>0.86651</v>
+        <v>0.8669</v>
       </c>
     </row>
   </sheetData>

</xml_diff>